<commit_message>
update: EventScoring.xlsx with Top CEO, Ultimate CEO, and Ultimate Traveler data
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/EventScoring.xlsx
+++ b/src/EventScoring.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mick/Documents/ApexGirl/CEO Calculators/src/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mick/Documents/ApexGirl/kts-unified/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A56DFE7-2BFA-3A41-B985-0E4CFE98B3C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F003F3A-F339-C74D-B70C-C218BC3C9F1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39480" yWindow="2640" windowWidth="32000" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1540" yWindow="2860" windowWidth="38880" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="78">
   <si>
     <t>TOP CEO EVENT</t>
   </si>
@@ -258,6 +258,15 @@
   </si>
   <si>
     <t>Promote Car x1</t>
+  </si>
+  <si>
+    <t>Ultimate Traveler</t>
+  </si>
+  <si>
+    <t>Slot Machine x1</t>
+  </si>
+  <si>
+    <t>Interview Artists x1</t>
   </si>
 </sst>
 </file>
@@ -354,7 +363,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -391,11 +400,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -459,22 +477,22 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -482,7 +500,19 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -817,7 +847,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q87"/>
+  <dimension ref="A1:W93"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" customWidth="1"/>
@@ -830,32 +860,42 @@
     <col min="13" max="13" width="7.83203125" customWidth="1"/>
     <col min="14" max="14" width="23.83203125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="7.83203125" customWidth="1"/>
+    <col min="20" max="20" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="29" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="24"/>
       <c r="D1" s="24"/>
       <c r="E1" s="24"/>
-      <c r="G1" s="23" t="s">
+      <c r="G1" s="29" t="s">
         <v>1</v>
       </c>
       <c r="H1" s="24"/>
       <c r="I1" s="24"/>
       <c r="J1" s="24"/>
       <c r="K1" s="24"/>
-      <c r="M1" s="23" t="s">
+      <c r="M1" s="29" t="s">
         <v>2</v>
       </c>
       <c r="N1" s="24"/>
       <c r="O1" s="24"/>
       <c r="P1" s="24"/>
       <c r="Q1" s="24"/>
-    </row>
-    <row r="2" spans="1:17" ht="6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S1" s="29" t="s">
+        <v>75</v>
+      </c>
+      <c r="T1" s="24"/>
+      <c r="U1" s="24"/>
+      <c r="V1" s="24"/>
+      <c r="W1" s="24"/>
+    </row>
+    <row r="2" spans="1:23" ht="6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="2"/>
       <c r="E2" s="4"/>
       <c r="F2" s="3"/>
@@ -866,29 +906,39 @@
       <c r="M2" s="2"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="5"/>
-    </row>
-    <row r="3" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R2" s="3"/>
+      <c r="S2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="5"/>
+    </row>
+    <row r="3" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="24"/>
-      <c r="N3" s="24"/>
-      <c r="O3" s="24"/>
-      <c r="P3" s="24"/>
-      <c r="Q3" s="32"/>
-    </row>
-    <row r="4" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="31"/>
+      <c r="N3" s="31"/>
+      <c r="O3" s="31"/>
+      <c r="P3" s="31"/>
+      <c r="Q3" s="31"/>
+      <c r="R3" s="31"/>
+      <c r="S3" s="31"/>
+      <c r="T3" s="31"/>
+      <c r="U3" s="31"/>
+      <c r="V3" s="31"/>
+      <c r="W3" s="31"/>
+    </row>
+    <row r="4" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="30" t="s">
         <v>0</v>
       </c>
@@ -899,20 +949,28 @@
       <c r="G4" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="24"/>
-      <c r="I4" s="24"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="5"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
       <c r="L4" s="3"/>
       <c r="M4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="N4" s="24"/>
-      <c r="O4" s="24"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="5"/>
-    </row>
-    <row r="5" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="N4" s="30"/>
+      <c r="O4" s="30"/>
+      <c r="P4" s="30"/>
+      <c r="Q4" s="30"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="T4" s="30"/>
+      <c r="U4" s="30"/>
+      <c r="V4" s="30"/>
+      <c r="W4" s="30"/>
+    </row>
+    <row r="5" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>4</v>
       </c>
@@ -926,6 +984,7 @@
         <v>7</v>
       </c>
       <c r="F5" s="6"/>
+      <c r="G5" s="2"/>
       <c r="H5" s="1" t="s">
         <v>4</v>
       </c>
@@ -951,9 +1010,22 @@
       <c r="Q5" s="7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="25" t="s">
+      <c r="R5" s="6"/>
+      <c r="T5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="V5" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="W5" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="26" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="9" t="s">
@@ -970,24 +1042,24 @@
         <v>0</v>
       </c>
       <c r="F6" s="10"/>
-      <c r="G6" s="25" t="s">
+      <c r="G6" s="26" t="s">
         <v>8</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I6" s="10">
-        <v>500</v>
+        <v>37500</v>
       </c>
       <c r="J6" s="10">
         <v>0</v>
       </c>
       <c r="K6" s="11">
-        <f t="shared" ref="K6:K15" si="1">J6*I6</f>
+        <f t="shared" ref="K6" si="1">J6*I6</f>
         <v>0</v>
       </c>
       <c r="L6" s="10"/>
-      <c r="M6" s="25" t="s">
+      <c r="M6" s="26" t="s">
         <v>9</v>
       </c>
       <c r="N6" s="9" t="s">
@@ -1003,8 +1075,25 @@
         <f t="shared" ref="Q6:Q22" si="2">P6*O6</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R6" s="10"/>
+      <c r="S6" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="T6" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="U6" s="10">
+        <v>500</v>
+      </c>
+      <c r="V6" s="10">
+        <v>0</v>
+      </c>
+      <c r="W6" s="11">
+        <f t="shared" ref="W6:W15" si="3">V6*U6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="24"/>
       <c r="B7" s="9" t="s">
         <v>74</v>
@@ -1020,18 +1109,18 @@
         <v>0</v>
       </c>
       <c r="F7" s="10"/>
-      <c r="G7" s="24"/>
+      <c r="G7" s="26"/>
       <c r="H7" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I7" s="10">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="J7" s="10">
         <v>0</v>
       </c>
       <c r="K7" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="K7:K16" si="4">J7*I7</f>
         <v>0</v>
       </c>
       <c r="L7" s="10"/>
@@ -1049,14 +1138,29 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R7" s="10"/>
+      <c r="S7" s="26"/>
+      <c r="T7" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="U7" s="10">
+        <v>2500</v>
+      </c>
+      <c r="V7" s="10">
+        <v>0</v>
+      </c>
+      <c r="W7" s="11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A8" s="24"/>
       <c r="B8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="C8" s="10">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="D8" s="10">
         <v>0</v>
@@ -1066,18 +1170,18 @@
         <v>0</v>
       </c>
       <c r="F8" s="10"/>
-      <c r="G8" s="24"/>
+      <c r="G8" s="26"/>
       <c r="H8" s="9" t="s">
-        <v>10</v>
+        <v>74</v>
       </c>
       <c r="I8" s="10">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="J8" s="10">
         <v>0</v>
       </c>
       <c r="K8" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="L8" s="10"/>
@@ -1095,14 +1199,29 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R8" s="10"/>
+      <c r="S8" s="26"/>
+      <c r="T8" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="U8" s="10">
+        <v>400</v>
+      </c>
+      <c r="V8" s="10">
+        <v>0</v>
+      </c>
+      <c r="W8" s="11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A9" s="24"/>
       <c r="B9" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C9" s="10">
-        <v>10000</v>
+        <v>50000</v>
       </c>
       <c r="D9" s="10">
         <v>0</v>
@@ -1112,18 +1231,18 @@
         <v>0</v>
       </c>
       <c r="F9" s="10"/>
-      <c r="G9" s="24"/>
+      <c r="G9" s="26"/>
       <c r="H9" s="9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I9" s="10">
-        <v>10000</v>
+        <v>400</v>
       </c>
       <c r="J9" s="10">
         <v>0</v>
       </c>
       <c r="K9" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="L9" s="10"/>
@@ -1141,11 +1260,26 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R9" s="10"/>
+      <c r="S9" s="26"/>
+      <c r="T9" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="U9" s="10">
+        <v>50000</v>
+      </c>
+      <c r="V9" s="10">
+        <v>0</v>
+      </c>
+      <c r="W9" s="11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A10" s="24"/>
       <c r="B10" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C10" s="10">
         <v>125000</v>
@@ -1158,18 +1292,18 @@
         <v>0</v>
       </c>
       <c r="F10" s="10"/>
-      <c r="G10" s="24"/>
+      <c r="G10" s="26"/>
       <c r="H10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="I10" s="10">
-        <v>125000</v>
+        <v>50000</v>
       </c>
       <c r="J10" s="10">
         <v>0</v>
       </c>
       <c r="K10" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="L10" s="10"/>
@@ -1187,14 +1321,29 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R10" s="10"/>
+      <c r="S10" s="26"/>
+      <c r="T10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="U10" s="10">
+        <v>6250000</v>
+      </c>
+      <c r="V10" s="10">
+        <v>0</v>
+      </c>
+      <c r="W10" s="11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A11" s="24"/>
       <c r="B11" s="9" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C11" s="10">
-        <v>1250000</v>
+        <v>4000</v>
       </c>
       <c r="D11" s="10">
         <v>0</v>
@@ -1204,18 +1353,18 @@
         <v>0</v>
       </c>
       <c r="F11" s="10"/>
-      <c r="G11" s="24"/>
+      <c r="G11" s="26"/>
       <c r="H11" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I11" s="10">
-        <v>1250000</v>
+        <v>6250000</v>
       </c>
       <c r="J11" s="10">
         <v>0</v>
       </c>
       <c r="K11" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="L11" s="10"/>
@@ -1233,14 +1382,29 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R11" s="10"/>
+      <c r="S11" s="26"/>
+      <c r="T11" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="U11" s="10">
+        <v>4000</v>
+      </c>
+      <c r="V11" s="10">
+        <v>0</v>
+      </c>
+      <c r="W11" s="11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12" s="24"/>
       <c r="B12" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C12" s="10">
-        <v>15625000</v>
+        <v>500000</v>
       </c>
       <c r="D12" s="10">
         <v>0</v>
@@ -1250,18 +1414,18 @@
         <v>0</v>
       </c>
       <c r="F12" s="10"/>
-      <c r="G12" s="24"/>
+      <c r="G12" s="26"/>
       <c r="H12" s="9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I12" s="10">
-        <v>15625000</v>
+        <v>4000</v>
       </c>
       <c r="J12" s="10">
         <v>0</v>
       </c>
       <c r="K12" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="L12" s="10"/>
@@ -1279,14 +1443,29 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R12" s="10"/>
+      <c r="S12" s="26"/>
+      <c r="T12" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="U12" s="10">
+        <v>500000</v>
+      </c>
+      <c r="V12" s="10">
+        <v>0</v>
+      </c>
+      <c r="W12" s="11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13" s="24"/>
       <c r="B13" s="9" t="s">
         <v>15</v>
       </c>
       <c r="C13" s="10">
-        <v>156250000</v>
+        <v>62500000</v>
       </c>
       <c r="D13" s="10">
         <v>0</v>
@@ -1296,18 +1475,18 @@
         <v>0</v>
       </c>
       <c r="F13" s="10"/>
-      <c r="G13" s="24"/>
+      <c r="G13" s="26"/>
       <c r="H13" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I13" s="10">
-        <v>156250000</v>
+        <v>500000</v>
       </c>
       <c r="J13" s="10">
         <v>0</v>
       </c>
       <c r="K13" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="L13" s="10"/>
@@ -1325,8 +1504,23 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R13" s="10"/>
+      <c r="S13" s="26"/>
+      <c r="T13" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="U13" s="10">
+        <v>62500000</v>
+      </c>
+      <c r="V13" s="10">
+        <v>0</v>
+      </c>
+      <c r="W13" s="11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A14" s="24"/>
       <c r="B14" s="9" t="s">
         <v>16</v>
@@ -1342,18 +1536,18 @@
         <v>0</v>
       </c>
       <c r="F14" s="10"/>
-      <c r="G14" s="24"/>
+      <c r="G14" s="26"/>
       <c r="H14" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I14" s="10">
-        <v>1</v>
+        <v>62500000</v>
       </c>
       <c r="J14" s="10">
         <v>0</v>
       </c>
       <c r="K14" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="L14" s="10"/>
@@ -1371,8 +1565,23 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R14" s="10"/>
+      <c r="S14" s="26"/>
+      <c r="T14" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="U14" s="10">
+        <v>1</v>
+      </c>
+      <c r="V14" s="10">
+        <v>0</v>
+      </c>
+      <c r="W14" s="11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A15" s="24"/>
       <c r="B15" s="9" t="s">
         <v>18</v>
@@ -1388,18 +1597,18 @@
         <v>0</v>
       </c>
       <c r="F15" s="10"/>
-      <c r="G15" s="24"/>
+      <c r="G15" s="26"/>
       <c r="H15" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I15" s="10">
-        <v>50000</v>
+        <v>1</v>
       </c>
       <c r="J15" s="10">
         <v>0</v>
       </c>
       <c r="K15" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="L15" s="10"/>
@@ -1417,8 +1626,23 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R15" s="10"/>
+      <c r="S15" s="26"/>
+      <c r="T15" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="U15" s="10">
+        <v>50000</v>
+      </c>
+      <c r="V15" s="10">
+        <v>0</v>
+      </c>
+      <c r="W15" s="11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A16" s="24"/>
       <c r="B16" s="9" t="s">
         <v>20</v>
@@ -1434,18 +1658,18 @@
         <v>0</v>
       </c>
       <c r="F16" s="10"/>
-      <c r="G16" s="24"/>
+      <c r="G16" s="26"/>
       <c r="H16" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I16" s="10">
-        <v>1</v>
+        <v>50000</v>
       </c>
       <c r="J16" s="10">
         <v>0</v>
       </c>
       <c r="K16" s="11">
-        <f>(J16*I16)/24</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="L16" s="10"/>
@@ -1463,8 +1687,23 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R16" s="10"/>
+      <c r="S16" s="26"/>
+      <c r="T16" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="U16" s="10">
+        <v>1</v>
+      </c>
+      <c r="V16" s="10">
+        <v>0</v>
+      </c>
+      <c r="W16" s="11">
+        <f>(V16*U16)/24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="24"/>
       <c r="B17" s="9" t="s">
         <v>22</v>
@@ -1480,18 +1719,18 @@
         <v>0</v>
       </c>
       <c r="F17" s="10"/>
-      <c r="G17" s="24"/>
+      <c r="G17" s="26"/>
       <c r="H17" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I17" s="10">
-        <v>10000</v>
+        <v>1</v>
       </c>
       <c r="J17" s="10">
         <v>0</v>
       </c>
       <c r="K17" s="11">
-        <f>J17*I17</f>
+        <f>(J17*I17)/24</f>
         <v>0</v>
       </c>
       <c r="L17" s="10"/>
@@ -1509,8 +1748,23 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R17" s="10"/>
+      <c r="S17" s="26"/>
+      <c r="T17" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="U17" s="10">
+        <v>10000</v>
+      </c>
+      <c r="V17" s="10">
+        <v>0</v>
+      </c>
+      <c r="W17" s="11">
+        <f>V17*U17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A18" s="24"/>
       <c r="B18" s="9" t="s">
         <v>24</v>
@@ -1526,12 +1780,12 @@
         <v>0</v>
       </c>
       <c r="F18" s="10"/>
-      <c r="G18" s="24"/>
+      <c r="G18" s="26"/>
       <c r="H18" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I18" s="10">
-        <v>40000</v>
+        <v>10000</v>
       </c>
       <c r="J18" s="10">
         <v>0</v>
@@ -1555,27 +1809,46 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R18" s="10"/>
+      <c r="S18" s="26"/>
+      <c r="T18" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="U18" s="10">
+        <v>40000</v>
+      </c>
+      <c r="V18" s="10">
+        <v>0</v>
+      </c>
+      <c r="W18" s="11">
+        <f>V18*U18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="12"/>
-      <c r="B19" s="26" t="s">
+      <c r="B19" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="27"/>
+      <c r="C19" s="25"/>
       <c r="D19" s="13"/>
       <c r="E19" s="14">
         <f>SUM(E6:E18)</f>
         <v>0</v>
       </c>
       <c r="F19" s="15"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="I19" s="27"/>
-      <c r="J19" s="13"/>
-      <c r="K19" s="14">
-        <f>SUM(K6:K18)</f>
+      <c r="G19" s="26"/>
+      <c r="H19" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="I19" s="10">
+        <v>40000</v>
+      </c>
+      <c r="J19" s="10">
+        <v>0</v>
+      </c>
+      <c r="K19" s="11">
+        <f>J19*I19</f>
         <v>0</v>
       </c>
       <c r="L19" s="15"/>
@@ -1593,9 +1866,24 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A20" s="25" t="s">
+      <c r="R19" s="15"/>
+      <c r="S19" s="26"/>
+      <c r="T19" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="U19" s="10">
+        <v>8</v>
+      </c>
+      <c r="V19" s="10">
+        <v>0</v>
+      </c>
+      <c r="W19" s="11">
+        <f>V19*U19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A20" s="26" t="s">
         <v>28</v>
       </c>
       <c r="B20" s="9" t="s">
@@ -1608,24 +1896,22 @@
         <v>0</v>
       </c>
       <c r="E20" s="16">
-        <f t="shared" ref="E20:E28" si="3">D20*C20</f>
+        <f t="shared" ref="E20:E28" si="5">D20*C20</f>
         <v>0</v>
       </c>
       <c r="F20" s="5"/>
-      <c r="G20" s="25" t="s">
-        <v>28</v>
-      </c>
+      <c r="G20" s="26"/>
       <c r="H20" s="9" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="I20" s="10">
-        <v>500</v>
+        <v>8</v>
       </c>
       <c r="J20" s="10">
         <v>0</v>
       </c>
-      <c r="K20" s="16">
-        <f t="shared" ref="K20:K28" si="4">J20*I20</f>
+      <c r="K20" s="11">
+        <f>J20*I20</f>
         <v>0</v>
       </c>
       <c r="L20" s="5"/>
@@ -1643,8 +1929,19 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R20" s="5"/>
+      <c r="S20" s="33"/>
+      <c r="T20" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="U20" s="25"/>
+      <c r="V20" s="13"/>
+      <c r="W20" s="14">
+        <f>SUM(W6:W19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="24"/>
       <c r="B21" s="9" t="s">
         <v>19</v>
@@ -1656,22 +1953,17 @@
         <v>0</v>
       </c>
       <c r="E21" s="16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="F21" s="5"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="I21" s="10">
-        <v>1000</v>
-      </c>
-      <c r="J21" s="10">
-        <v>0</v>
-      </c>
-      <c r="K21" s="16">
-        <f t="shared" si="4"/>
+      <c r="H21" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="I21" s="25"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="14">
+        <f>SUM(K7:K19)</f>
         <v>0</v>
       </c>
       <c r="L21" s="5"/>
@@ -1689,8 +1981,25 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R21" s="5"/>
+      <c r="S21" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="T21" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="U21" s="10">
+        <v>500</v>
+      </c>
+      <c r="V21" s="10">
+        <v>0</v>
+      </c>
+      <c r="W21" s="11">
+        <f t="shared" ref="W21:W29" si="6">V21*U21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="24"/>
       <c r="B22" s="9" t="s">
         <v>25</v>
@@ -1702,22 +2011,24 @@
         <v>0</v>
       </c>
       <c r="E22" s="16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="F22" s="5"/>
-      <c r="G22" s="24"/>
+      <c r="G22" s="26" t="s">
+        <v>28</v>
+      </c>
       <c r="H22" s="9" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="I22" s="10">
-        <v>10000</v>
+        <v>37500</v>
       </c>
       <c r="J22" s="10">
         <v>0</v>
       </c>
-      <c r="K22" s="16">
-        <f t="shared" si="4"/>
+      <c r="K22" s="11">
+        <f t="shared" ref="K22" si="7">J22*I22</f>
         <v>0</v>
       </c>
       <c r="L22" s="5"/>
@@ -1735,8 +2046,23 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R22" s="5"/>
+      <c r="S22" s="26"/>
+      <c r="T22" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="U22" s="10">
+        <v>400</v>
+      </c>
+      <c r="V22" s="10">
+        <v>0</v>
+      </c>
+      <c r="W22" s="11">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A23" s="24"/>
       <c r="B23" s="9" t="s">
         <v>21</v>
@@ -1748,22 +2074,22 @@
         <v>0</v>
       </c>
       <c r="E23" s="16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="F23" s="5"/>
-      <c r="G23" s="24"/>
+      <c r="G23" s="26"/>
       <c r="H23" s="9" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I23" s="10">
-        <v>125000</v>
+        <v>500</v>
       </c>
       <c r="J23" s="10">
         <v>0</v>
       </c>
       <c r="K23" s="16">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="K23:K31" si="8">J23*I23</f>
         <v>0</v>
       </c>
       <c r="L23" s="5"/>
@@ -1781,8 +2107,23 @@
         <f>(P23*O23)/24</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R23" s="5"/>
+      <c r="S23" s="26"/>
+      <c r="T23" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="U23" s="10">
+        <v>50000</v>
+      </c>
+      <c r="V23" s="10">
+        <v>0</v>
+      </c>
+      <c r="W23" s="11">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A24" s="24"/>
       <c r="B24" s="9" t="s">
         <v>27</v>
@@ -1794,22 +2135,22 @@
         <v>0</v>
       </c>
       <c r="E24" s="16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="F24" s="5"/>
-      <c r="G24" s="24"/>
+      <c r="G24" s="26"/>
       <c r="H24" s="9" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="I24" s="10">
-        <v>1250000</v>
+        <v>400</v>
       </c>
       <c r="J24" s="10">
         <v>0</v>
       </c>
       <c r="K24" s="16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="L24" s="5"/>
@@ -1827,8 +2168,23 @@
         <f>P24*O24</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R24" s="5"/>
+      <c r="S24" s="26"/>
+      <c r="T24" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="U24" s="10">
+        <v>6250000</v>
+      </c>
+      <c r="V24" s="10">
+        <v>0</v>
+      </c>
+      <c r="W24" s="11">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A25" s="24"/>
       <c r="B25" s="9" t="s">
         <v>23</v>
@@ -1840,22 +2196,22 @@
         <v>0</v>
       </c>
       <c r="E25" s="16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="F25" s="5"/>
-      <c r="G25" s="24"/>
+      <c r="G25" s="26"/>
       <c r="H25" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I25" s="10">
-        <v>15625000</v>
+        <v>4000</v>
       </c>
       <c r="J25" s="10">
         <v>0</v>
       </c>
       <c r="K25" s="16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="L25" s="5"/>
@@ -1873,8 +2229,23 @@
         <f>P25*O25</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R25" s="5"/>
+      <c r="S25" s="26"/>
+      <c r="T25" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="U25" s="10">
+        <v>4000</v>
+      </c>
+      <c r="V25" s="10">
+        <v>0</v>
+      </c>
+      <c r="W25" s="11">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A26" s="24"/>
       <c r="B26" s="9" t="s">
         <v>29</v>
@@ -1886,22 +2257,22 @@
         <v>0</v>
       </c>
       <c r="E26" s="16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="F26" s="5"/>
-      <c r="G26" s="24"/>
+      <c r="G26" s="26"/>
       <c r="H26" s="9" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="I26" s="10">
-        <v>156250000</v>
+        <v>50000</v>
       </c>
       <c r="J26" s="10">
         <v>0</v>
       </c>
       <c r="K26" s="16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="L26" s="5"/>
@@ -1919,8 +2290,23 @@
         <f>P26*O26</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R26" s="5"/>
+      <c r="S26" s="26"/>
+      <c r="T26" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="U26" s="10">
+        <v>500000</v>
+      </c>
+      <c r="V26" s="10">
+        <v>0</v>
+      </c>
+      <c r="W26" s="11">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A27" s="24"/>
       <c r="B27" s="9" t="s">
         <v>16</v>
@@ -1932,36 +2318,51 @@
         <v>0</v>
       </c>
       <c r="E27" s="16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="F27" s="5"/>
-      <c r="G27" s="24"/>
+      <c r="G27" s="26"/>
       <c r="H27" s="9" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="I27" s="10">
-        <v>1</v>
+        <v>500000</v>
       </c>
       <c r="J27" s="10">
         <v>0</v>
       </c>
       <c r="K27" s="16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="L27" s="5"/>
-      <c r="N27" s="26" t="s">
+      <c r="N27" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="O27" s="27"/>
+      <c r="O27" s="25"/>
       <c r="P27" s="13"/>
       <c r="Q27" s="14">
         <f>SUM(Q6:Q26)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R27" s="5"/>
+      <c r="S27" s="26"/>
+      <c r="T27" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="U27" s="10">
+        <v>62500000</v>
+      </c>
+      <c r="V27" s="10">
+        <v>0</v>
+      </c>
+      <c r="W27" s="11">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A28" s="24"/>
       <c r="B28" s="9" t="s">
         <v>18</v>
@@ -1973,26 +2374,26 @@
         <v>0</v>
       </c>
       <c r="E28" s="16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="F28" s="5"/>
-      <c r="G28" s="24"/>
+      <c r="G28" s="26"/>
       <c r="H28" s="9" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="I28" s="10">
-        <v>50000</v>
+        <v>6250000</v>
       </c>
       <c r="J28" s="10">
         <v>0</v>
       </c>
       <c r="K28" s="16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="L28" s="5"/>
-      <c r="M28" s="25" t="s">
+      <c r="M28" s="26" t="s">
         <v>31</v>
       </c>
       <c r="N28" s="9" t="s">
@@ -2005,11 +2406,26 @@
         <v>0</v>
       </c>
       <c r="Q28" s="16">
-        <f t="shared" ref="Q28:Q45" si="5">O28*P28</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" ref="Q28:Q45" si="9">O28*P28</f>
+        <v>0</v>
+      </c>
+      <c r="R28" s="5"/>
+      <c r="S28" s="26"/>
+      <c r="T28" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="U28" s="10">
+        <v>1</v>
+      </c>
+      <c r="V28" s="10">
+        <v>0</v>
+      </c>
+      <c r="W28" s="11">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A29" s="24"/>
       <c r="B29" s="9" t="s">
         <v>20</v>
@@ -2025,18 +2441,18 @@
         <v>0</v>
       </c>
       <c r="F29" s="5"/>
-      <c r="G29" s="24"/>
+      <c r="G29" s="26"/>
       <c r="H29" s="9" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="I29" s="10">
-        <v>1</v>
+        <v>62500000</v>
       </c>
       <c r="J29" s="10">
         <v>0</v>
       </c>
       <c r="K29" s="16">
-        <f>J29*I29/24</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="L29" s="5"/>
@@ -2051,11 +2467,26 @@
         <v>0</v>
       </c>
       <c r="Q29" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R29" s="5"/>
+      <c r="S29" s="26"/>
+      <c r="T29" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="U29" s="10">
+        <v>50000</v>
+      </c>
+      <c r="V29" s="10">
+        <v>0</v>
+      </c>
+      <c r="W29" s="11">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="24"/>
       <c r="B30" s="9" t="s">
         <v>22</v>
@@ -2071,18 +2502,18 @@
         <v>0</v>
       </c>
       <c r="F30" s="5"/>
-      <c r="G30" s="24"/>
+      <c r="G30" s="26"/>
       <c r="H30" s="9" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="I30" s="10">
-        <v>10000</v>
+        <v>1</v>
       </c>
       <c r="J30" s="10">
         <v>0</v>
       </c>
       <c r="K30" s="16">
-        <f>J30*I30</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="L30" s="5"/>
@@ -2097,11 +2528,26 @@
         <v>0</v>
       </c>
       <c r="Q30" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R30" s="5"/>
+      <c r="S30" s="26"/>
+      <c r="T30" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="U30" s="10">
+        <v>1</v>
+      </c>
+      <c r="V30" s="10">
+        <v>0</v>
+      </c>
+      <c r="W30" s="11">
+        <f>(V30*U30)/24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A31" s="24"/>
       <c r="B31" s="9" t="s">
         <v>24</v>
@@ -2117,18 +2563,18 @@
         <v>0</v>
       </c>
       <c r="F31" s="5"/>
-      <c r="G31" s="24"/>
+      <c r="G31" s="26"/>
       <c r="H31" s="9" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="I31" s="10">
-        <v>40000</v>
+        <v>50000</v>
       </c>
       <c r="J31" s="10">
         <v>0</v>
       </c>
       <c r="K31" s="16">
-        <f>J31*I31</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="L31" s="5"/>
@@ -2143,30 +2589,49 @@
         <v>0</v>
       </c>
       <c r="Q31" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R31" s="5"/>
+      <c r="S31" s="26"/>
+      <c r="T31" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="U31" s="10">
+        <v>10000</v>
+      </c>
+      <c r="V31" s="10">
+        <v>0</v>
+      </c>
+      <c r="W31" s="11">
+        <f>V31*U31</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="17"/>
-      <c r="B32" s="26" t="s">
+      <c r="B32" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C32" s="27"/>
+      <c r="C32" s="25"/>
       <c r="D32" s="13"/>
       <c r="E32" s="18">
         <f>SUM(E20:E31)</f>
         <v>0</v>
       </c>
       <c r="F32" s="19"/>
-      <c r="G32" s="17"/>
-      <c r="H32" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="I32" s="27"/>
-      <c r="J32" s="13"/>
-      <c r="K32" s="18">
-        <f>SUM(K20:K31)</f>
+      <c r="G32" s="26"/>
+      <c r="H32" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="I32" s="10">
+        <v>1</v>
+      </c>
+      <c r="J32" s="10">
+        <v>0</v>
+      </c>
+      <c r="K32" s="16">
+        <f>J32*I32/24</f>
         <v>0</v>
       </c>
       <c r="L32" s="19"/>
@@ -2181,12 +2646,27 @@
         <v>0</v>
       </c>
       <c r="Q32" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A33" s="25" t="s">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R32" s="19"/>
+      <c r="S32" s="26"/>
+      <c r="T32" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="U32" s="10">
+        <v>40000</v>
+      </c>
+      <c r="V32" s="10">
+        <v>0</v>
+      </c>
+      <c r="W32" s="11">
+        <f>V32*U32</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A33" s="26" t="s">
         <v>37</v>
       </c>
       <c r="B33" s="9" t="s">
@@ -2199,24 +2679,22 @@
         <v>0</v>
       </c>
       <c r="E33" s="16">
-        <f t="shared" ref="E33:E42" si="6">C33*D33</f>
+        <f t="shared" ref="E33:E42" si="10">C33*D33</f>
         <v>0</v>
       </c>
       <c r="F33" s="5"/>
-      <c r="G33" s="25" t="s">
-        <v>37</v>
-      </c>
+      <c r="G33" s="26"/>
       <c r="H33" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="I33" s="20">
-        <v>500</v>
+        <v>22</v>
+      </c>
+      <c r="I33" s="10">
+        <v>10000</v>
       </c>
       <c r="J33" s="10">
         <v>0</v>
       </c>
       <c r="K33" s="16">
-        <f t="shared" ref="K33:K42" si="7">I33*J33</f>
+        <f>J33*I33</f>
         <v>0</v>
       </c>
       <c r="L33" s="5"/>
@@ -2231,11 +2709,26 @@
         <v>0</v>
       </c>
       <c r="Q33" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R33" s="5"/>
+      <c r="S33" s="26"/>
+      <c r="T33" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="U33" s="10">
+        <v>8</v>
+      </c>
+      <c r="V33" s="10">
+        <v>0</v>
+      </c>
+      <c r="W33" s="11">
+        <f>V33*U33</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A34" s="24"/>
       <c r="B34" s="9" t="s">
         <v>33</v>
@@ -2247,22 +2740,22 @@
         <v>0</v>
       </c>
       <c r="E34" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F34" s="5"/>
-      <c r="G34" s="24"/>
+      <c r="G34" s="26"/>
       <c r="H34" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="I34" s="20">
-        <v>1000</v>
+        <v>24</v>
+      </c>
+      <c r="I34" s="10">
+        <v>40000</v>
       </c>
       <c r="J34" s="10">
         <v>0</v>
       </c>
       <c r="K34" s="16">
-        <f t="shared" si="7"/>
+        <f>J34*I34</f>
         <v>0</v>
       </c>
       <c r="L34" s="5"/>
@@ -2277,11 +2770,22 @@
         <v>0</v>
       </c>
       <c r="Q34" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R34" s="5"/>
+      <c r="S34" s="33"/>
+      <c r="T34" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="U34" s="25"/>
+      <c r="V34" s="13"/>
+      <c r="W34" s="14">
+        <f>SUM(W21:W33)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="24"/>
       <c r="B35" s="9" t="s">
         <v>34</v>
@@ -2293,22 +2797,22 @@
         <v>0</v>
       </c>
       <c r="E35" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F35" s="5"/>
-      <c r="G35" s="24"/>
+      <c r="G35" s="26"/>
       <c r="H35" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="I35" s="9">
-        <v>2000</v>
+        <v>30</v>
+      </c>
+      <c r="I35" s="10">
+        <v>8</v>
       </c>
       <c r="J35" s="10">
         <v>0</v>
       </c>
-      <c r="K35" s="16">
-        <f t="shared" si="7"/>
+      <c r="K35" s="11">
+        <f>J35*I35</f>
         <v>0</v>
       </c>
       <c r="L35" s="5"/>
@@ -2323,11 +2827,28 @@
         <v>0</v>
       </c>
       <c r="Q35" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R35" s="5"/>
+      <c r="S35" s="26" t="s">
+        <v>37</v>
+      </c>
+      <c r="T35" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="U35" s="20">
+        <v>500</v>
+      </c>
+      <c r="V35" s="10">
+        <v>0</v>
+      </c>
+      <c r="W35" s="16">
+        <f t="shared" ref="W35:W44" si="11">U35*V35</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="24"/>
       <c r="B36" s="9" t="s">
         <v>38</v>
@@ -2339,22 +2860,18 @@
         <v>0</v>
       </c>
       <c r="E36" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F36" s="5"/>
-      <c r="G36" s="24"/>
-      <c r="H36" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="I36">
-        <v>20000</v>
-      </c>
-      <c r="J36" s="10">
-        <v>0</v>
-      </c>
-      <c r="K36" s="16">
-        <f t="shared" si="7"/>
+      <c r="G36" s="36"/>
+      <c r="H36" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="I36" s="25"/>
+      <c r="J36" s="13"/>
+      <c r="K36" s="18">
+        <f>SUM(K23:K34)</f>
         <v>0</v>
       </c>
       <c r="L36" s="5"/>
@@ -2369,11 +2886,26 @@
         <v>0</v>
       </c>
       <c r="Q36" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R36" s="5"/>
+      <c r="S36" s="26"/>
+      <c r="T36" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="U36" s="20">
+        <v>1000</v>
+      </c>
+      <c r="V36" s="10">
+        <v>0</v>
+      </c>
+      <c r="W36" s="16">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A37" s="24"/>
       <c r="B37" s="9" t="s">
         <v>35</v>
@@ -2385,22 +2917,22 @@
         <v>0</v>
       </c>
       <c r="E37" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F37" s="5"/>
-      <c r="G37" s="24"/>
+      <c r="G37" s="8"/>
       <c r="H37" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="I37">
-        <v>250000</v>
+        <v>76</v>
+      </c>
+      <c r="I37" s="10">
+        <v>37500</v>
       </c>
       <c r="J37" s="10">
         <v>0</v>
       </c>
-      <c r="K37" s="16">
-        <f t="shared" si="7"/>
+      <c r="K37" s="11">
+        <f t="shared" ref="K37" si="12">J37*I37</f>
         <v>0</v>
       </c>
       <c r="L37" s="5"/>
@@ -2415,11 +2947,26 @@
         <v>0</v>
       </c>
       <c r="Q37" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R37" s="5"/>
+      <c r="S37" s="26"/>
+      <c r="T37" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="U37" s="9">
+        <v>400</v>
+      </c>
+      <c r="V37" s="10">
+        <v>0</v>
+      </c>
+      <c r="W37" s="16">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A38" s="24"/>
       <c r="B38" s="9" t="s">
         <v>39</v>
@@ -2431,22 +2978,24 @@
         <v>0</v>
       </c>
       <c r="E38" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F38" s="5"/>
-      <c r="G38" s="24"/>
+      <c r="G38" s="26" t="s">
+        <v>37</v>
+      </c>
       <c r="H38" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="I38">
-        <v>2500000</v>
+        <v>32</v>
+      </c>
+      <c r="I38" s="20">
+        <v>500</v>
       </c>
       <c r="J38" s="10">
         <v>0</v>
       </c>
       <c r="K38" s="16">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="K38:K47" si="13">I38*J38</f>
         <v>0</v>
       </c>
       <c r="L38" s="5"/>
@@ -2461,11 +3010,26 @@
         <v>0</v>
       </c>
       <c r="Q38" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R38" s="5"/>
+      <c r="S38" s="26"/>
+      <c r="T38" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="U38" s="9">
+        <v>50000</v>
+      </c>
+      <c r="V38" s="10">
+        <v>0</v>
+      </c>
+      <c r="W38" s="16">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A39" s="24"/>
       <c r="B39" s="9" t="s">
         <v>36</v>
@@ -2477,22 +3041,22 @@
         <v>0</v>
       </c>
       <c r="E39" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F39" s="5"/>
-      <c r="G39" s="24"/>
+      <c r="G39" s="26"/>
       <c r="H39" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="I39">
-        <v>31250000</v>
+        <v>33</v>
+      </c>
+      <c r="I39" s="20">
+        <v>1000</v>
       </c>
       <c r="J39" s="10">
         <v>0</v>
       </c>
       <c r="K39" s="16">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L39" s="5"/>
@@ -2507,11 +3071,26 @@
         <v>0</v>
       </c>
       <c r="Q39" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R39" s="5"/>
+      <c r="S39" s="26"/>
+      <c r="T39" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="U39" s="9">
+        <v>6250000</v>
+      </c>
+      <c r="V39" s="10">
+        <v>0</v>
+      </c>
+      <c r="W39" s="16">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A40" s="24"/>
       <c r="B40" s="9" t="s">
         <v>40</v>
@@ -2523,22 +3102,22 @@
         <v>0</v>
       </c>
       <c r="E40" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F40" s="5"/>
-      <c r="G40" s="24"/>
+      <c r="G40" s="26"/>
       <c r="H40" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="I40">
-        <v>312500000</v>
+        <v>34</v>
+      </c>
+      <c r="I40" s="9">
+        <v>1000</v>
       </c>
       <c r="J40" s="10">
         <v>0</v>
       </c>
       <c r="K40" s="16">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L40" s="5"/>
@@ -2553,11 +3132,26 @@
         <v>0</v>
       </c>
       <c r="Q40" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R40" s="5"/>
+      <c r="S40" s="26"/>
+      <c r="T40" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="U40" s="9">
+        <v>4000</v>
+      </c>
+      <c r="V40" s="10">
+        <v>0</v>
+      </c>
+      <c r="W40" s="16">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A41" s="24"/>
       <c r="B41" s="9" t="s">
         <v>16</v>
@@ -2569,22 +3163,22 @@
         <v>0</v>
       </c>
       <c r="E41" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F41" s="5"/>
-      <c r="G41" s="24"/>
+      <c r="G41" s="26"/>
       <c r="H41" s="9" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="I41">
-        <v>1</v>
+        <v>10000</v>
       </c>
       <c r="J41" s="10">
         <v>0</v>
       </c>
       <c r="K41" s="16">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L41" s="5"/>
@@ -2599,11 +3193,26 @@
         <v>0</v>
       </c>
       <c r="Q41" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R41" s="5"/>
+      <c r="S41" s="26"/>
+      <c r="T41" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="U41" s="9">
+        <v>500000</v>
+      </c>
+      <c r="V41" s="10">
+        <v>0</v>
+      </c>
+      <c r="W41" s="16">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A42" s="24"/>
       <c r="B42" s="9" t="s">
         <v>18</v>
@@ -2615,22 +3224,22 @@
         <v>0</v>
       </c>
       <c r="E42" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F42" s="5"/>
-      <c r="G42" s="24"/>
+      <c r="G42" s="26"/>
       <c r="H42" s="9" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="I42">
-        <v>50000</v>
+        <v>125000</v>
       </c>
       <c r="J42" s="10">
         <v>0</v>
       </c>
       <c r="K42" s="16">
-        <f t="shared" si="7"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L42" s="5"/>
@@ -2645,11 +3254,26 @@
         <v>0</v>
       </c>
       <c r="Q42" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R42" s="5"/>
+      <c r="S42" s="26"/>
+      <c r="T42" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="U42" s="9">
+        <v>62500000</v>
+      </c>
+      <c r="V42" s="10">
+        <v>0</v>
+      </c>
+      <c r="W42" s="16">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A43" s="24"/>
       <c r="B43" s="9" t="s">
         <v>20</v>
@@ -2665,18 +3289,18 @@
         <v>0</v>
       </c>
       <c r="F43" s="5"/>
-      <c r="G43" s="24"/>
+      <c r="G43" s="26"/>
       <c r="H43" s="9" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="I43">
-        <v>1</v>
+        <v>1250000</v>
       </c>
       <c r="J43" s="10">
         <v>0</v>
       </c>
       <c r="K43" s="16">
-        <f>(I43*J43)/24</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L43" s="5"/>
@@ -2691,11 +3315,26 @@
         <v>0</v>
       </c>
       <c r="Q43" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R43" s="5"/>
+      <c r="S43" s="26"/>
+      <c r="T43" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="U43">
+        <v>1</v>
+      </c>
+      <c r="V43" s="10">
+        <v>0</v>
+      </c>
+      <c r="W43" s="16">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="24"/>
       <c r="B44" s="9" t="s">
         <v>22</v>
@@ -2711,18 +3350,18 @@
         <v>0</v>
       </c>
       <c r="F44" s="5"/>
-      <c r="G44" s="24"/>
+      <c r="G44" s="26"/>
       <c r="H44" s="9" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="I44">
-        <v>10000</v>
+        <v>15625000</v>
       </c>
       <c r="J44" s="10">
         <v>0</v>
       </c>
       <c r="K44" s="16">
-        <f>I44*J44</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L44" s="5"/>
@@ -2737,11 +3376,26 @@
         <v>0</v>
       </c>
       <c r="Q44" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R44" s="5"/>
+      <c r="S44" s="26"/>
+      <c r="T44" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="U44">
+        <v>50000</v>
+      </c>
+      <c r="V44" s="10">
+        <v>0</v>
+      </c>
+      <c r="W44" s="16">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A45" s="24"/>
       <c r="B45" s="9" t="s">
         <v>24</v>
@@ -2757,18 +3411,18 @@
         <v>0</v>
       </c>
       <c r="F45" s="5"/>
-      <c r="G45" s="24"/>
+      <c r="G45" s="26"/>
       <c r="H45" s="9" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="I45">
-        <v>40000</v>
+        <v>156250000</v>
       </c>
       <c r="J45" s="10">
         <v>0</v>
       </c>
       <c r="K45" s="16">
-        <f>I45*J45</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L45" s="5"/>
@@ -2783,30 +3437,49 @@
         <v>0</v>
       </c>
       <c r="Q45" s="16">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="R45" s="5"/>
+      <c r="S45" s="26"/>
+      <c r="T45" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="U45">
+        <v>1</v>
+      </c>
+      <c r="V45" s="10">
+        <v>0</v>
+      </c>
+      <c r="W45" s="16">
+        <f>(U45*V45)/24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="13"/>
-      <c r="B46" s="26" t="s">
+      <c r="B46" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="C46" s="27"/>
+      <c r="C46" s="25"/>
       <c r="D46" s="13"/>
       <c r="E46" s="18">
         <f>SUM(E33:E45)</f>
         <v>0</v>
       </c>
       <c r="F46" s="19"/>
-      <c r="G46" s="13"/>
-      <c r="H46" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="I46" s="27"/>
-      <c r="J46" s="13"/>
-      <c r="K46" s="18">
-        <f>SUM(K33:K45)</f>
+      <c r="G46" s="26"/>
+      <c r="H46" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I46">
+        <v>1</v>
+      </c>
+      <c r="J46" s="10">
+        <v>0</v>
+      </c>
+      <c r="K46" s="16">
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L46" s="19"/>
@@ -2824,9 +3497,24 @@
         <f>(O46*P46)/24</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A47" s="29" t="s">
+      <c r="R46" s="19"/>
+      <c r="S46" s="26"/>
+      <c r="T46" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="U46">
+        <v>10000</v>
+      </c>
+      <c r="V46" s="10">
+        <v>0</v>
+      </c>
+      <c r="W46" s="16">
+        <f>U46*V46</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A47" s="28" t="s">
         <v>50</v>
       </c>
       <c r="B47" s="9" t="s">
@@ -2839,24 +3527,22 @@
         <v>0</v>
       </c>
       <c r="E47" s="16">
-        <f t="shared" ref="E47:E57" si="8">D47*C47</f>
+        <f t="shared" ref="E47:E57" si="14">D47*C47</f>
         <v>0</v>
       </c>
       <c r="F47" s="5"/>
-      <c r="G47" s="29" t="s">
-        <v>50</v>
-      </c>
+      <c r="G47" s="26"/>
       <c r="H47" s="9" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="I47">
-        <v>37500</v>
-      </c>
-      <c r="J47" s="5">
+        <v>50000</v>
+      </c>
+      <c r="J47" s="10">
         <v>0</v>
       </c>
       <c r="K47" s="16">
-        <f t="shared" ref="K47:K57" si="9">J47*I47</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L47" s="5"/>
@@ -2874,8 +3560,23 @@
         <f>O47*P47</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R47" s="5"/>
+      <c r="S47" s="26"/>
+      <c r="T47" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="U47">
+        <v>40000</v>
+      </c>
+      <c r="V47" s="10">
+        <v>0</v>
+      </c>
+      <c r="W47" s="16">
+        <f>U47*V47</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A48" s="24"/>
       <c r="B48" s="9" t="s">
         <v>41</v>
@@ -2887,22 +3588,22 @@
         <v>0</v>
       </c>
       <c r="E48" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F48" s="5"/>
-      <c r="G48" s="24"/>
+      <c r="G48" s="26"/>
       <c r="H48" s="9" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="I48">
-        <v>500</v>
-      </c>
-      <c r="J48" s="5">
+        <v>1</v>
+      </c>
+      <c r="J48" s="10">
         <v>0</v>
       </c>
       <c r="K48" s="16">
-        <f t="shared" si="9"/>
+        <f>(I48*J48)/24</f>
         <v>0</v>
       </c>
       <c r="L48" s="5"/>
@@ -2920,8 +3621,23 @@
         <f>O48*P48</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R48" s="5"/>
+      <c r="S48" s="26"/>
+      <c r="T48" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="U48">
+        <v>8</v>
+      </c>
+      <c r="V48" s="10">
+        <v>0</v>
+      </c>
+      <c r="W48" s="16">
+        <f>U48*V48</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A49" s="24"/>
       <c r="B49" s="9" t="s">
         <v>42</v>
@@ -2933,22 +3649,22 @@
         <v>0</v>
       </c>
       <c r="E49" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F49" s="5"/>
-      <c r="G49" s="24"/>
+      <c r="G49" s="26"/>
       <c r="H49" s="9" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="I49">
-        <v>5000</v>
-      </c>
-      <c r="J49" s="5">
+        <v>10000</v>
+      </c>
+      <c r="J49" s="10">
         <v>0</v>
       </c>
       <c r="K49" s="16">
-        <f t="shared" si="9"/>
+        <f>I49*J49</f>
         <v>0</v>
       </c>
       <c r="L49" s="5"/>
@@ -2966,8 +3682,19 @@
         <f>O49*P49</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R49" s="5"/>
+      <c r="S49" s="32"/>
+      <c r="T49" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="U49" s="25"/>
+      <c r="V49" s="13"/>
+      <c r="W49" s="18">
+        <f>SUM(W35:W48)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="24"/>
       <c r="B50" s="9" t="s">
         <v>52</v>
@@ -2979,36 +3706,53 @@
         <v>0</v>
       </c>
       <c r="E50" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F50" s="5"/>
-      <c r="G50" s="24"/>
+      <c r="G50" s="26"/>
       <c r="H50" s="9" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="I50">
-        <v>2000</v>
-      </c>
-      <c r="J50" s="5">
+        <v>40000</v>
+      </c>
+      <c r="J50" s="10">
         <v>0</v>
       </c>
       <c r="K50" s="16">
-        <f t="shared" si="9"/>
+        <f>I50*J50</f>
         <v>0</v>
       </c>
       <c r="L50" s="5"/>
-      <c r="N50" s="26" t="s">
+      <c r="N50" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="O50" s="27"/>
+      <c r="O50" s="25"/>
       <c r="P50" s="13"/>
       <c r="Q50" s="18">
         <f>SUM(Q28:Q49)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R50" s="5"/>
+      <c r="S50" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="T50" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="U50" s="9">
+        <v>500</v>
+      </c>
+      <c r="V50" s="10">
+        <v>0</v>
+      </c>
+      <c r="W50" s="16">
+        <f t="shared" ref="W50:W59" si="15">U50*V50</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A51" s="24"/>
       <c r="B51" s="9" t="s">
         <v>46</v>
@@ -3020,26 +3764,26 @@
         <v>0</v>
       </c>
       <c r="E51" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F51" s="5"/>
-      <c r="G51" s="24"/>
+      <c r="G51" s="26"/>
       <c r="H51" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="I51">
-        <v>20000</v>
-      </c>
-      <c r="J51" s="5">
-        <v>0</v>
-      </c>
-      <c r="K51" s="16">
-        <f t="shared" si="9"/>
+        <v>30</v>
+      </c>
+      <c r="I51" s="10">
+        <v>8</v>
+      </c>
+      <c r="J51" s="10">
+        <v>0</v>
+      </c>
+      <c r="K51" s="11">
+        <f>J51*I51</f>
         <v>0</v>
       </c>
       <c r="L51" s="5"/>
-      <c r="M51" s="25" t="s">
+      <c r="M51" s="26" t="s">
         <v>53</v>
       </c>
       <c r="N51" s="9" t="s">
@@ -3052,11 +3796,26 @@
         <v>0</v>
       </c>
       <c r="Q51" s="16">
-        <f t="shared" ref="Q51:Q59" si="10">O51*P51</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" ref="Q51:Q59" si="16">O51*P51</f>
+        <v>0</v>
+      </c>
+      <c r="R51" s="5"/>
+      <c r="S51" s="26"/>
+      <c r="T51" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="U51" s="9">
+        <v>5000</v>
+      </c>
+      <c r="V51" s="10">
+        <v>0</v>
+      </c>
+      <c r="W51" s="16">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A52" s="24"/>
       <c r="B52" s="9" t="s">
         <v>55</v>
@@ -3068,22 +3827,18 @@
         <v>0</v>
       </c>
       <c r="E52" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F52" s="5"/>
-      <c r="G52" s="24"/>
-      <c r="H52" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="I52">
-        <v>250000</v>
-      </c>
-      <c r="J52" s="5">
-        <v>0</v>
-      </c>
-      <c r="K52" s="16">
-        <f t="shared" si="9"/>
+      <c r="G52" s="13"/>
+      <c r="H52" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="I52" s="25"/>
+      <c r="J52" s="13"/>
+      <c r="K52" s="18">
+        <f>SUM(K38:K50)</f>
         <v>0</v>
       </c>
       <c r="L52" s="5"/>
@@ -3098,11 +3853,26 @@
         <v>0</v>
       </c>
       <c r="Q52" s="16">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="R52" s="5"/>
+      <c r="S52" s="26"/>
+      <c r="T52" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="U52" s="9">
+        <v>1000</v>
+      </c>
+      <c r="V52" s="10">
+        <v>0</v>
+      </c>
+      <c r="W52" s="16">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="24"/>
       <c r="B53" s="9" t="s">
         <v>47</v>
@@ -3114,22 +3884,24 @@
         <v>0</v>
       </c>
       <c r="E53" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F53" s="5"/>
-      <c r="G53" s="24"/>
+      <c r="G53" s="34" t="s">
+        <v>50</v>
+      </c>
       <c r="H53" s="9" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="I53">
-        <v>2500000</v>
+        <v>500</v>
       </c>
       <c r="J53" s="5">
         <v>0</v>
       </c>
       <c r="K53" s="16">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="K53:K62" si="17">J53*I53</f>
         <v>0</v>
       </c>
       <c r="L53" s="5"/>
@@ -3144,11 +3916,26 @@
         <v>0</v>
       </c>
       <c r="Q53" s="16">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="R53" s="5"/>
+      <c r="S53" s="26"/>
+      <c r="T53" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="U53" s="9">
+        <v>125000</v>
+      </c>
+      <c r="V53" s="10">
+        <v>0</v>
+      </c>
+      <c r="W53" s="16">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A54" s="24"/>
       <c r="B54" s="9" t="s">
         <v>58</v>
@@ -3160,22 +3947,22 @@
         <v>0</v>
       </c>
       <c r="E54" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F54" s="5"/>
-      <c r="G54" s="24"/>
+      <c r="G54" s="35"/>
       <c r="H54" s="9" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="I54">
-        <v>31250000</v>
+        <v>5000</v>
       </c>
       <c r="J54" s="5">
         <v>0</v>
       </c>
       <c r="K54" s="16">
-        <f t="shared" si="9"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="L54" s="5"/>
@@ -3190,11 +3977,26 @@
         <v>0</v>
       </c>
       <c r="Q54" s="16">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="R54" s="5"/>
+      <c r="S54" s="26"/>
+      <c r="T54" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="U54">
+        <v>15625000</v>
+      </c>
+      <c r="V54" s="10">
+        <v>0</v>
+      </c>
+      <c r="W54" s="16">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A55" s="24"/>
       <c r="B55" s="9" t="s">
         <v>48</v>
@@ -3206,22 +4008,22 @@
         <v>0</v>
       </c>
       <c r="E55" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F55" s="5"/>
-      <c r="G55" s="24"/>
+      <c r="G55" s="35"/>
       <c r="H55" s="9" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I55">
-        <v>312500000</v>
+        <v>1000</v>
       </c>
       <c r="J55" s="5">
         <v>0</v>
       </c>
       <c r="K55" s="16">
-        <f t="shared" si="9"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="L55" s="5"/>
@@ -3236,11 +4038,26 @@
         <v>0</v>
       </c>
       <c r="Q55" s="16">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="R55" s="5"/>
+      <c r="S55" s="26"/>
+      <c r="T55" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="U55">
+        <v>10000</v>
+      </c>
+      <c r="V55" s="10">
+        <v>0</v>
+      </c>
+      <c r="W55" s="16">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="24"/>
       <c r="B56" s="9" t="s">
         <v>16</v>
@@ -3252,22 +4069,22 @@
         <v>0</v>
       </c>
       <c r="E56" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F56" s="5"/>
-      <c r="G56" s="24"/>
+      <c r="G56" s="35"/>
       <c r="H56" s="9" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="I56">
-        <v>1</v>
+        <v>10000</v>
       </c>
       <c r="J56" s="5">
         <v>0</v>
       </c>
       <c r="K56" s="16">
-        <f t="shared" si="9"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="L56" s="5"/>
@@ -3282,11 +4099,26 @@
         <v>0</v>
       </c>
       <c r="Q56" s="16">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="R56" s="5"/>
+      <c r="S56" s="26"/>
+      <c r="T56" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="U56">
+        <v>1250000</v>
+      </c>
+      <c r="V56" s="10">
+        <v>0</v>
+      </c>
+      <c r="W56" s="16">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A57" s="24"/>
       <c r="B57" s="9" t="s">
         <v>18</v>
@@ -3298,22 +4130,22 @@
         <v>0</v>
       </c>
       <c r="E57" s="16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F57" s="5"/>
-      <c r="G57" s="24"/>
+      <c r="G57" s="35"/>
       <c r="H57" s="9" t="s">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="I57">
-        <v>50000</v>
+        <v>125000</v>
       </c>
       <c r="J57" s="5">
         <v>0</v>
       </c>
       <c r="K57" s="16">
-        <f t="shared" si="9"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="L57" s="5"/>
@@ -3328,11 +4160,26 @@
         <v>0</v>
       </c>
       <c r="Q57" s="16">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="R57" s="5"/>
+      <c r="S57" s="26"/>
+      <c r="T57" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="U57">
+        <v>156250000</v>
+      </c>
+      <c r="V57" s="10">
+        <v>0</v>
+      </c>
+      <c r="W57" s="16">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A58" s="24"/>
       <c r="B58" s="9" t="s">
         <v>20</v>
@@ -3348,18 +4195,18 @@
         <v>0</v>
       </c>
       <c r="F58" s="5"/>
-      <c r="G58" s="24"/>
+      <c r="G58" s="35"/>
       <c r="H58" s="9" t="s">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="I58">
-        <v>1</v>
+        <v>1250000</v>
       </c>
       <c r="J58" s="5">
         <v>0</v>
       </c>
       <c r="K58" s="16">
-        <f>(J58*I58)/24</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="L58" s="5"/>
@@ -3374,12 +4221,27 @@
         <v>0</v>
       </c>
       <c r="Q58" s="16">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="27"/>
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="R58" s="5"/>
+      <c r="S58" s="26"/>
+      <c r="T58" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="U58">
+        <v>1</v>
+      </c>
+      <c r="V58" s="10">
+        <v>0</v>
+      </c>
+      <c r="W58" s="16">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="25"/>
       <c r="B59" s="9" t="s">
         <v>22</v>
       </c>
@@ -3394,18 +4256,18 @@
         <v>0</v>
       </c>
       <c r="F59" s="5"/>
-      <c r="G59" s="27"/>
+      <c r="G59" s="35"/>
       <c r="H59" s="9" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
       <c r="I59">
-        <v>10000</v>
+        <v>15625000</v>
       </c>
       <c r="J59" s="5">
         <v>0</v>
       </c>
       <c r="K59" s="16">
-        <f>J59*I59</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="L59" s="5"/>
@@ -3420,11 +4282,26 @@
         <v>0</v>
       </c>
       <c r="Q59" s="16">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.2">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="R59" s="5"/>
+      <c r="S59" s="26"/>
+      <c r="T59" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="U59">
+        <v>50000</v>
+      </c>
+      <c r="V59" s="10">
+        <v>0</v>
+      </c>
+      <c r="W59" s="16">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A60" s="8"/>
       <c r="B60" s="9" t="s">
         <v>24</v>
@@ -3440,18 +4317,18 @@
         <v>0</v>
       </c>
       <c r="F60" s="5"/>
-      <c r="G60" s="8"/>
+      <c r="G60" s="35"/>
       <c r="H60" s="9" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="I60">
-        <v>40000</v>
+        <v>156250000</v>
       </c>
       <c r="J60" s="5">
         <v>0</v>
       </c>
       <c r="K60" s="16">
-        <f>J60*I60</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="L60" s="5"/>
@@ -3469,27 +4346,46 @@
         <f>(O60*P60)/24</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R60" s="5"/>
+      <c r="S60" s="26"/>
+      <c r="T60" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="U60">
+        <v>1</v>
+      </c>
+      <c r="V60" s="10">
+        <v>0</v>
+      </c>
+      <c r="W60" s="16">
+        <f>(U60*V60)/24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="13"/>
-      <c r="B61" s="26" t="s">
+      <c r="B61" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="C61" s="27"/>
+      <c r="C61" s="25"/>
       <c r="D61" s="13"/>
       <c r="E61" s="18">
         <f>SUM(E47:E60)</f>
         <v>0</v>
       </c>
       <c r="F61" s="19"/>
-      <c r="G61" s="13"/>
-      <c r="H61" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="I61" s="27"/>
-      <c r="J61" s="13"/>
-      <c r="K61" s="18">
-        <f>SUM(K47:K60)</f>
+      <c r="G61" s="35"/>
+      <c r="H61" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I61">
+        <v>1</v>
+      </c>
+      <c r="J61" s="5">
+        <v>0</v>
+      </c>
+      <c r="K61" s="16">
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="L61" s="19"/>
@@ -3507,9 +4403,24 @@
         <f>O61*P61</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A62" s="25" t="s">
+      <c r="R61" s="19"/>
+      <c r="S61" s="26"/>
+      <c r="T61" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="U61">
+        <v>10000</v>
+      </c>
+      <c r="V61" s="10">
+        <v>0</v>
+      </c>
+      <c r="W61" s="16">
+        <f>U61*V61</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A62" s="26" t="s">
         <v>63</v>
       </c>
       <c r="B62" s="9" t="s">
@@ -3522,24 +4433,22 @@
         <v>0</v>
       </c>
       <c r="E62" s="16">
-        <f t="shared" ref="E62:E69" si="11">D62*C62</f>
+        <f t="shared" ref="E62:E69" si="18">D62*C62</f>
         <v>0</v>
       </c>
       <c r="F62" s="5"/>
-      <c r="G62" s="25" t="s">
-        <v>63</v>
-      </c>
+      <c r="G62" s="35"/>
       <c r="H62" s="9" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="I62">
-        <v>37500</v>
+        <v>50000</v>
       </c>
       <c r="J62" s="5">
         <v>0</v>
       </c>
       <c r="K62" s="16">
-        <f t="shared" ref="K62:K69" si="12">J62*I62</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="L62" s="5"/>
@@ -3557,8 +4466,23 @@
         <f>O62*P62</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R62" s="5"/>
+      <c r="S62" s="26"/>
+      <c r="T62" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="U62">
+        <v>40000</v>
+      </c>
+      <c r="V62" s="10">
+        <v>0</v>
+      </c>
+      <c r="W62" s="16">
+        <f>U62*V62</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A63" s="24"/>
       <c r="B63" s="9" t="s">
         <v>64</v>
@@ -3570,22 +4494,22 @@
         <v>0</v>
       </c>
       <c r="E63" s="16">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="F63" s="5"/>
-      <c r="G63" s="24"/>
+      <c r="G63" s="35"/>
       <c r="H63" s="9" t="s">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="I63">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J63" s="5">
         <v>0</v>
       </c>
       <c r="K63" s="16">
-        <f t="shared" si="12"/>
+        <f>(J63*I63)/24</f>
         <v>0</v>
       </c>
       <c r="L63" s="5"/>
@@ -3603,8 +4527,23 @@
         <f>O63*P63</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R63" s="5"/>
+      <c r="S63" s="26"/>
+      <c r="T63" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="U63">
+        <v>8</v>
+      </c>
+      <c r="V63" s="10">
+        <v>0</v>
+      </c>
+      <c r="W63" s="16">
+        <f>U63*V63</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A64" s="24"/>
       <c r="B64" s="9" t="s">
         <v>59</v>
@@ -3616,36 +4555,47 @@
         <v>0</v>
       </c>
       <c r="E64" s="16">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="F64" s="5"/>
-      <c r="G64" s="24"/>
+      <c r="G64" s="35"/>
       <c r="H64" s="9" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="I64">
-        <v>1500</v>
+        <v>10000</v>
       </c>
       <c r="J64" s="5">
         <v>0</v>
       </c>
       <c r="K64" s="16">
-        <f t="shared" si="12"/>
+        <f>J64*I64</f>
         <v>0</v>
       </c>
       <c r="L64" s="5"/>
-      <c r="N64" s="26" t="s">
+      <c r="N64" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="O64" s="27"/>
+      <c r="O64" s="25"/>
       <c r="P64" s="5"/>
       <c r="Q64" s="21">
         <f>SUM(Q51:Q63)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R64" s="5"/>
+      <c r="S64" s="32"/>
+      <c r="T64" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="U64" s="25"/>
+      <c r="V64" s="13"/>
+      <c r="W64" s="18">
+        <f>SUM(W50:W63)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A65" s="24"/>
       <c r="B65" s="9" t="s">
         <v>60</v>
@@ -3657,33 +4607,50 @@
         <v>0</v>
       </c>
       <c r="E65" s="16">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="F65" s="5"/>
-      <c r="G65" s="24"/>
+      <c r="G65" s="35"/>
       <c r="H65" s="9" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="I65">
-        <v>4000</v>
+        <v>40000</v>
       </c>
       <c r="J65" s="5">
         <v>0</v>
       </c>
       <c r="K65" s="16">
-        <f t="shared" si="12"/>
+        <f>J65*I65</f>
         <v>0</v>
       </c>
       <c r="L65" s="5"/>
-      <c r="N65" s="28" t="s">
+      <c r="N65" s="23" t="s">
         <v>65</v>
       </c>
       <c r="O65" s="24"/>
       <c r="P65" s="24"/>
       <c r="Q65" s="16"/>
-    </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R65" s="5"/>
+      <c r="S65" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="T65" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="U65" s="9">
+        <v>5</v>
+      </c>
+      <c r="V65" s="10">
+        <v>0</v>
+      </c>
+      <c r="W65" s="16">
+        <f t="shared" ref="W65:W71" si="19">U65*V65</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A66" s="24"/>
       <c r="B66" s="9" t="s">
         <v>66</v>
@@ -3695,34 +4662,49 @@
         <v>0</v>
       </c>
       <c r="E66" s="16">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="F66" s="5"/>
-      <c r="G66" s="24"/>
+      <c r="G66" s="35"/>
       <c r="H66" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="I66">
-        <v>4000</v>
-      </c>
-      <c r="J66" s="5">
-        <v>0</v>
-      </c>
-      <c r="K66" s="16">
-        <f t="shared" si="12"/>
+        <v>30</v>
+      </c>
+      <c r="I66" s="10">
+        <v>8</v>
+      </c>
+      <c r="J66" s="10">
+        <v>0</v>
+      </c>
+      <c r="K66" s="11">
+        <f>J66*I66</f>
         <v>0</v>
       </c>
       <c r="L66" s="5"/>
-      <c r="N66" s="27"/>
-      <c r="O66" s="27"/>
-      <c r="P66" s="27"/>
+      <c r="N66" s="25"/>
+      <c r="O66" s="25"/>
+      <c r="P66" s="25"/>
       <c r="Q66" s="11">
         <f>SUM(Q64+Q50+Q27)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R66" s="5"/>
+      <c r="S66" s="26"/>
+      <c r="T66" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="U66" s="9">
+        <v>1500</v>
+      </c>
+      <c r="V66" s="10">
+        <v>0</v>
+      </c>
+      <c r="W66" s="16">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A67" s="24"/>
       <c r="B67" s="9" t="s">
         <v>67</v>
@@ -3734,27 +4716,38 @@
         <v>0</v>
       </c>
       <c r="E67" s="16">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="F67" s="5"/>
-      <c r="G67" s="24"/>
-      <c r="H67" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="I67">
-        <v>25000</v>
-      </c>
-      <c r="J67" s="5">
-        <v>0</v>
-      </c>
-      <c r="K67" s="16">
-        <f t="shared" si="12"/>
+      <c r="G67" s="13"/>
+      <c r="H67" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="I67" s="27"/>
+      <c r="J67" s="13"/>
+      <c r="K67" s="18">
+        <f>SUM(K53:K65)</f>
         <v>0</v>
       </c>
       <c r="L67" s="5"/>
-    </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R67" s="5"/>
+      <c r="S67" s="26"/>
+      <c r="T67" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="U67" s="9">
+        <v>4000</v>
+      </c>
+      <c r="V67" s="10">
+        <v>0</v>
+      </c>
+      <c r="W67" s="16">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="24"/>
       <c r="B68" s="9" t="s">
         <v>16</v>
@@ -3766,27 +4759,44 @@
         <v>0</v>
       </c>
       <c r="E68" s="16">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="F68" s="5"/>
-      <c r="G68" s="24"/>
+      <c r="G68" s="34" t="s">
+        <v>63</v>
+      </c>
       <c r="H68" s="9" t="s">
-        <v>16</v>
+        <v>64</v>
       </c>
       <c r="I68">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J68" s="5">
         <v>0</v>
       </c>
       <c r="K68" s="16">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="K68:K74" si="20">J68*I68</f>
         <v>0</v>
       </c>
       <c r="L68" s="5"/>
-    </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R68" s="5"/>
+      <c r="S68" s="26"/>
+      <c r="T68" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="U68" s="9">
+        <v>4000</v>
+      </c>
+      <c r="V68" s="10">
+        <v>0</v>
+      </c>
+      <c r="W68" s="16">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A69" s="24"/>
       <c r="B69" s="9" t="s">
         <v>18</v>
@@ -3798,27 +4808,42 @@
         <v>0</v>
       </c>
       <c r="E69" s="16">
-        <f t="shared" si="11"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="F69" s="5"/>
-      <c r="G69" s="24"/>
+      <c r="G69" s="26"/>
       <c r="H69" s="9" t="s">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="I69">
-        <v>50000</v>
+        <v>1500</v>
       </c>
       <c r="J69" s="5">
         <v>0</v>
       </c>
       <c r="K69" s="16">
-        <f t="shared" si="12"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="L69" s="5"/>
-    </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R69" s="5"/>
+      <c r="S69" s="26"/>
+      <c r="T69" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="U69" s="9">
+        <v>25000</v>
+      </c>
+      <c r="V69" s="10">
+        <v>0</v>
+      </c>
+      <c r="W69" s="16">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A70" s="24"/>
       <c r="B70" s="9" t="s">
         <v>20</v>
@@ -3834,23 +4859,38 @@
         <v>0</v>
       </c>
       <c r="F70" s="5"/>
-      <c r="G70" s="24"/>
+      <c r="G70" s="26"/>
       <c r="H70" s="9" t="s">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="I70">
+        <v>4000</v>
+      </c>
+      <c r="J70" s="5">
+        <v>0</v>
+      </c>
+      <c r="K70" s="16">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="L70" s="5"/>
+      <c r="R70" s="5"/>
+      <c r="S70" s="26"/>
+      <c r="T70" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="U70">
         <v>1</v>
       </c>
-      <c r="J70" s="5">
-        <v>0</v>
-      </c>
-      <c r="K70" s="16">
-        <f>(J70*I70)/24</f>
-        <v>0</v>
-      </c>
-      <c r="L70" s="5"/>
-    </row>
-    <row r="71" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V70" s="10">
+        <v>0</v>
+      </c>
+      <c r="W70" s="16">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="24"/>
       <c r="B71" s="9" t="s">
         <v>22</v>
@@ -3866,23 +4906,38 @@
         <v>0</v>
       </c>
       <c r="F71" s="5"/>
-      <c r="G71" s="24"/>
+      <c r="G71" s="26"/>
       <c r="H71" s="9" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="I71">
-        <v>10000</v>
+        <v>4000</v>
       </c>
       <c r="J71" s="5">
         <v>0</v>
       </c>
       <c r="K71" s="16">
-        <f>J71*I71</f>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="L71" s="5"/>
-    </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R71" s="5"/>
+      <c r="S71" s="26"/>
+      <c r="T71" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="U71">
+        <v>50000</v>
+      </c>
+      <c r="V71" s="10">
+        <v>0</v>
+      </c>
+      <c r="W71" s="16">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A72" s="24"/>
       <c r="B72" s="9" t="s">
         <v>24</v>
@@ -3898,46 +4953,81 @@
         <v>0</v>
       </c>
       <c r="F72" s="5"/>
-      <c r="G72" s="24"/>
+      <c r="G72" s="26"/>
       <c r="H72" s="9" t="s">
-        <v>24</v>
+        <v>67</v>
       </c>
       <c r="I72">
-        <v>40000</v>
+        <v>25000</v>
       </c>
       <c r="J72" s="5">
         <v>0</v>
       </c>
       <c r="K72" s="16">
-        <f>J72*I72</f>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="L72" s="5"/>
-    </row>
-    <row r="73" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B73" s="26" t="s">
+      <c r="R72" s="5"/>
+      <c r="S72" s="26"/>
+      <c r="T72" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="U72">
+        <v>1</v>
+      </c>
+      <c r="V72" s="10">
+        <v>0</v>
+      </c>
+      <c r="W72" s="16">
+        <f>(U72*V72)/24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B73" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="C73" s="27"/>
+      <c r="C73" s="25"/>
       <c r="D73" s="5"/>
       <c r="E73" s="21">
         <f>SUM(E62:E72)</f>
         <v>0</v>
       </c>
       <c r="F73" s="22"/>
-      <c r="H73" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="I73" s="27"/>
-      <c r="J73" s="5"/>
-      <c r="K73" s="21">
-        <f>SUM(K62:K72)</f>
+      <c r="G73" s="26"/>
+      <c r="H73" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I73">
+        <v>1</v>
+      </c>
+      <c r="J73" s="5">
+        <v>0</v>
+      </c>
+      <c r="K73" s="16">
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="L73" s="22"/>
-    </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A74" s="25" t="s">
+      <c r="R73" s="22"/>
+      <c r="S73" s="26"/>
+      <c r="T73" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="U73">
+        <v>10000</v>
+      </c>
+      <c r="V73" s="10">
+        <v>0</v>
+      </c>
+      <c r="W73" s="16">
+        <f>U73*V73</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A74" s="26" t="s">
         <v>68</v>
       </c>
       <c r="B74" s="9" t="s">
@@ -3950,29 +5040,42 @@
         <v>0</v>
       </c>
       <c r="E74" s="16">
-        <f t="shared" ref="E74:E84" si="13">D74*C74</f>
+        <f t="shared" ref="E74:E84" si="21">D74*C74</f>
         <v>0</v>
       </c>
       <c r="F74" s="5"/>
-      <c r="G74" s="25" t="s">
-        <v>68</v>
-      </c>
+      <c r="G74" s="26"/>
       <c r="H74" s="9" t="s">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="I74">
-        <v>12</v>
+        <v>50000</v>
       </c>
       <c r="J74" s="5">
         <v>0</v>
       </c>
       <c r="K74" s="16">
-        <f t="shared" ref="K74:K84" si="14">J74*I74</f>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="L74" s="5"/>
-    </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R74" s="5"/>
+      <c r="S74" s="26"/>
+      <c r="T74" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="U74">
+        <v>40000</v>
+      </c>
+      <c r="V74" s="10">
+        <v>0</v>
+      </c>
+      <c r="W74" s="16">
+        <f>U74*V74</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A75" s="24"/>
       <c r="B75" s="9" t="s">
         <v>70</v>
@@ -3984,27 +5087,42 @@
         <v>0</v>
       </c>
       <c r="E75" s="16">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="F75" s="5"/>
-      <c r="G75" s="24"/>
+      <c r="G75" s="26"/>
       <c r="H75" s="9" t="s">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="I75">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="J75" s="5">
         <v>0</v>
       </c>
       <c r="K75" s="16">
-        <f t="shared" si="14"/>
+        <f>(J75*I75)/24</f>
         <v>0</v>
       </c>
       <c r="L75" s="5"/>
-    </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R75" s="5"/>
+      <c r="S75" s="26"/>
+      <c r="T75" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="U75">
+        <v>8</v>
+      </c>
+      <c r="V75" s="10">
+        <v>0</v>
+      </c>
+      <c r="W75" s="16">
+        <f>U75*V75</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A76" s="24"/>
       <c r="B76" s="9" t="s">
         <v>51</v>
@@ -4016,27 +5134,38 @@
         <v>0</v>
       </c>
       <c r="E76" s="16">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="F76" s="5"/>
-      <c r="G76" s="24"/>
+      <c r="G76" s="26"/>
       <c r="H76" s="9" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="I76">
-        <v>37500</v>
+        <v>10000</v>
       </c>
       <c r="J76" s="5">
         <v>0</v>
       </c>
       <c r="K76" s="16">
-        <f t="shared" si="14"/>
+        <f>J76*I76</f>
         <v>0</v>
       </c>
       <c r="L76" s="5"/>
-    </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R76" s="5"/>
+      <c r="S76" s="32"/>
+      <c r="T76" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="U76" s="25"/>
+      <c r="V76" s="5"/>
+      <c r="W76" s="21">
+        <f>SUM(W65:W75)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A77" s="24"/>
       <c r="B77" s="9" t="s">
         <v>20</v>
@@ -4048,27 +5177,35 @@
         <v>0</v>
       </c>
       <c r="E77" s="16">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="F77" s="5"/>
-      <c r="G77" s="24"/>
+      <c r="G77" s="26"/>
       <c r="H77" s="9" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I77">
-        <v>1</v>
+        <v>40000</v>
       </c>
       <c r="J77" s="5">
         <v>0</v>
       </c>
       <c r="K77" s="16">
-        <f t="shared" si="14"/>
+        <f>J77*I77</f>
         <v>0</v>
       </c>
       <c r="L77" s="5"/>
-    </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R77" s="5"/>
+      <c r="S77" s="8"/>
+      <c r="T77" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="U77" s="24"/>
+      <c r="V77" s="24"/>
+      <c r="W77" s="16"/>
+    </row>
+    <row r="78" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A78" s="24"/>
       <c r="B78" s="9" t="s">
         <v>18</v>
@@ -4080,27 +5217,35 @@
         <v>0</v>
       </c>
       <c r="E78" s="16">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="F78" s="5"/>
-      <c r="G78" s="24"/>
+      <c r="G78" s="26"/>
       <c r="H78" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="I78">
-        <v>50000</v>
-      </c>
-      <c r="J78" s="5">
-        <v>0</v>
-      </c>
-      <c r="K78" s="16">
-        <f t="shared" si="14"/>
+        <v>30</v>
+      </c>
+      <c r="I78" s="10">
+        <v>8</v>
+      </c>
+      <c r="J78" s="10">
+        <v>0</v>
+      </c>
+      <c r="K78" s="11">
+        <f>J78*I78</f>
         <v>0</v>
       </c>
       <c r="L78" s="5"/>
-    </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R78" s="5"/>
+      <c r="T78" s="25"/>
+      <c r="U78" s="25"/>
+      <c r="V78" s="25"/>
+      <c r="W78" s="11">
+        <f>SUM(W76+W63+W20)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A79" s="24"/>
       <c r="B79" s="9" t="s">
         <v>16</v>
@@ -4112,27 +5257,26 @@
         <v>0</v>
       </c>
       <c r="E79" s="16">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="F79" s="5"/>
-      <c r="G79" s="24"/>
+      <c r="G79" s="26"/>
       <c r="H79" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="I79">
-        <v>1</v>
-      </c>
-      <c r="J79" s="5">
-        <v>0</v>
-      </c>
-      <c r="K79" s="16">
-        <f t="shared" si="14"/>
+        <v>77</v>
+      </c>
+      <c r="I79" s="10">
+        <v>60000</v>
+      </c>
+      <c r="J79" s="10"/>
+      <c r="K79" s="11">
+        <f>J79*I79</f>
         <v>0</v>
       </c>
       <c r="L79" s="5"/>
-    </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R79" s="5"/>
+    </row>
+    <row r="80" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A80" s="24"/>
       <c r="B80" s="9" t="s">
         <v>22</v>
@@ -4144,27 +5288,23 @@
         <v>0</v>
       </c>
       <c r="E80" s="16">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="F80" s="5"/>
-      <c r="G80" s="24"/>
-      <c r="H80" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I80">
-        <v>10000</v>
-      </c>
-      <c r="J80" s="5">
-        <v>0</v>
-      </c>
-      <c r="K80" s="16">
-        <f t="shared" si="14"/>
+      <c r="H80" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="I80" s="25"/>
+      <c r="J80" s="5"/>
+      <c r="K80" s="21">
+        <f>SUM(K68:K77)</f>
         <v>0</v>
       </c>
       <c r="L80" s="5"/>
-    </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="R80" s="5"/>
+    </row>
+    <row r="81" spans="1:18" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="24"/>
       <c r="B81" s="9" t="s">
         <v>24</v>
@@ -4176,27 +5316,30 @@
         <v>0</v>
       </c>
       <c r="E81" s="16">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="F81" s="5"/>
-      <c r="G81" s="24"/>
+      <c r="G81" s="26" t="s">
+        <v>68</v>
+      </c>
       <c r="H81" s="9" t="s">
-        <v>24</v>
+        <v>69</v>
       </c>
       <c r="I81">
-        <v>40000</v>
+        <v>12</v>
       </c>
       <c r="J81" s="5">
         <v>0</v>
       </c>
       <c r="K81" s="16">
-        <f t="shared" si="14"/>
+        <f t="shared" ref="K81:K90" si="22">J81*I81</f>
         <v>0</v>
       </c>
       <c r="L81" s="5"/>
-    </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="R81" s="5"/>
+    </row>
+    <row r="82" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A82" s="24"/>
       <c r="B82" s="9" t="s">
         <v>71</v>
@@ -4208,27 +5351,28 @@
         <v>0</v>
       </c>
       <c r="E82" s="16">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="F82" s="5"/>
-      <c r="G82" s="24"/>
+      <c r="G82" s="26"/>
       <c r="H82" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I82">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J82" s="5">
         <v>0</v>
       </c>
       <c r="K82" s="16">
-        <f t="shared" si="14"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="L82" s="5"/>
-    </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="R82" s="5"/>
+    </row>
+    <row r="83" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A83" s="24"/>
       <c r="B83" s="9" t="s">
         <v>72</v>
@@ -4240,27 +5384,28 @@
         <v>0</v>
       </c>
       <c r="E83" s="16">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="F83" s="5"/>
-      <c r="G83" s="24"/>
+      <c r="G83" s="26"/>
       <c r="H83" s="9" t="s">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="I83">
-        <v>500</v>
+        <v>1</v>
       </c>
       <c r="J83" s="5">
         <v>0</v>
       </c>
       <c r="K83" s="16">
-        <f t="shared" si="14"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="L83" s="5"/>
-    </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="R83" s="5"/>
+    </row>
+    <row r="84" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A84" s="24"/>
       <c r="B84" s="9" t="s">
         <v>54</v>
@@ -4272,130 +5417,248 @@
         <v>0</v>
       </c>
       <c r="E84" s="16">
-        <f t="shared" si="13"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="F84" s="5"/>
-      <c r="G84" s="24"/>
+      <c r="G84" s="26"/>
       <c r="H84" s="9" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="I84">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="J84" s="5">
         <v>0</v>
       </c>
       <c r="K84" s="16">
-        <f t="shared" si="14"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="L84" s="5"/>
-    </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B85" s="26" t="s">
+      <c r="R84" s="5"/>
+    </row>
+    <row r="85" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B85" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="C85" s="27"/>
+      <c r="C85" s="25"/>
       <c r="D85" s="5"/>
       <c r="E85" s="16">
         <f>SUM(E74:E84)</f>
         <v>0</v>
       </c>
       <c r="F85" s="5"/>
-      <c r="H85" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="I85" s="27"/>
-      <c r="J85" s="5"/>
+      <c r="G85" s="26"/>
+      <c r="H85" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I85">
+        <v>1</v>
+      </c>
+      <c r="J85" s="5">
+        <v>0</v>
+      </c>
       <c r="K85" s="16">
-        <f>SUM(K74:K84)</f>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="L85" s="5"/>
-    </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B86" s="28" t="s">
+      <c r="R85" s="5"/>
+    </row>
+    <row r="86" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B86" s="23" t="s">
         <v>65</v>
       </c>
       <c r="C86" s="24"/>
       <c r="D86" s="24"/>
       <c r="E86" s="16"/>
       <c r="F86" s="5"/>
-      <c r="H86" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="I86" s="24"/>
-      <c r="J86" s="24"/>
-      <c r="K86" s="16"/>
+      <c r="G86" s="26"/>
+      <c r="H86" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="I86">
+        <v>10000</v>
+      </c>
+      <c r="J86" s="5">
+        <v>0</v>
+      </c>
+      <c r="K86" s="16">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
       <c r="L86" s="5"/>
-    </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B87" s="27"/>
-      <c r="C87" s="27"/>
-      <c r="D87" s="27"/>
+      <c r="R86" s="5"/>
+    </row>
+    <row r="87" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B87" s="25"/>
+      <c r="C87" s="25"/>
+      <c r="D87" s="25"/>
       <c r="E87" s="11">
         <f>SUM(E85+E73+E61+E46+E32+E19)</f>
         <v>0</v>
       </c>
       <c r="F87" s="10"/>
-      <c r="H87" s="27"/>
-      <c r="I87" s="27"/>
-      <c r="J87" s="27"/>
-      <c r="K87" s="11">
-        <f>SUM(K85+K73+K61+K46+K32+K19)</f>
+      <c r="G87" s="26"/>
+      <c r="H87" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="I87">
+        <v>40000</v>
+      </c>
+      <c r="J87" s="5">
+        <v>0</v>
+      </c>
+      <c r="K87" s="16">
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="L87" s="10"/>
+      <c r="R87" s="10"/>
+    </row>
+    <row r="88" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="G88" s="26"/>
+      <c r="H88" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="I88">
+        <v>8</v>
+      </c>
+      <c r="J88" s="5">
+        <v>0</v>
+      </c>
+      <c r="K88" s="16">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="G89" s="26"/>
+      <c r="H89" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="I89">
+        <v>500</v>
+      </c>
+      <c r="J89" s="5">
+        <v>0</v>
+      </c>
+      <c r="K89" s="16">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="G90" s="26"/>
+      <c r="H90" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="I90">
+        <v>60000</v>
+      </c>
+      <c r="J90" s="5">
+        <v>0</v>
+      </c>
+      <c r="K90" s="16">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="G91" s="32"/>
+      <c r="H91" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="I91" s="25"/>
+      <c r="J91" s="5"/>
+      <c r="K91" s="16">
+        <f>SUM(K81:K90)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="H92" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="I92" s="24"/>
+      <c r="J92" s="24"/>
+      <c r="K92" s="16"/>
+    </row>
+    <row r="93" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="H93" s="25"/>
+      <c r="I93" s="25"/>
+      <c r="J93" s="25"/>
+      <c r="K93" s="11">
+        <f>SUM(K91+K80+K67+K52+K36+K21)</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="40">
-    <mergeCell ref="N65:P66"/>
-    <mergeCell ref="A74:A84"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="A6:A18"/>
-    <mergeCell ref="G62:G72"/>
-    <mergeCell ref="A33:A45"/>
-    <mergeCell ref="A62:A72"/>
-    <mergeCell ref="A20:A31"/>
-    <mergeCell ref="A47:A59"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="M6:M26"/>
-    <mergeCell ref="N50:O50"/>
-    <mergeCell ref="M51:M63"/>
-    <mergeCell ref="N27:O27"/>
-    <mergeCell ref="B86:D87"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="G47:G59"/>
-    <mergeCell ref="H86:J87"/>
-    <mergeCell ref="M1:Q1"/>
-    <mergeCell ref="H73:I73"/>
-    <mergeCell ref="H46:I46"/>
-    <mergeCell ref="G74:G84"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="G6:G18"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="N64:O64"/>
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="M4:O4"/>
+  <mergeCells count="53">
+    <mergeCell ref="T76:U76"/>
+    <mergeCell ref="T77:V78"/>
+    <mergeCell ref="S6:S19"/>
+    <mergeCell ref="T34:U34"/>
+    <mergeCell ref="S21:S33"/>
+    <mergeCell ref="T49:U49"/>
+    <mergeCell ref="T64:U64"/>
+    <mergeCell ref="S35:S48"/>
+    <mergeCell ref="S50:S63"/>
+    <mergeCell ref="S65:S75"/>
+    <mergeCell ref="S1:W1"/>
+    <mergeCell ref="T20:U20"/>
+    <mergeCell ref="A3:W3"/>
+    <mergeCell ref="G6:G20"/>
+    <mergeCell ref="G4:K4"/>
+    <mergeCell ref="M4:Q4"/>
+    <mergeCell ref="S4:W4"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="G1:K1"/>
     <mergeCell ref="M28:M48"/>
     <mergeCell ref="B85:C85"/>
     <mergeCell ref="B32:C32"/>
-    <mergeCell ref="G20:G31"/>
-    <mergeCell ref="H85:I85"/>
-    <mergeCell ref="G33:G45"/>
-    <mergeCell ref="H61:I61"/>
+    <mergeCell ref="H91:I91"/>
+    <mergeCell ref="H67:I67"/>
     <mergeCell ref="B4:D4"/>
+    <mergeCell ref="G38:G51"/>
+    <mergeCell ref="G22:G35"/>
+    <mergeCell ref="G53:G66"/>
+    <mergeCell ref="G68:G79"/>
+    <mergeCell ref="G81:G90"/>
+    <mergeCell ref="B86:D87"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="H92:J93"/>
+    <mergeCell ref="M1:Q1"/>
+    <mergeCell ref="H80:I80"/>
+    <mergeCell ref="H52:I52"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="N64:O64"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="N65:P66"/>
+    <mergeCell ref="A74:A84"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="A6:A18"/>
+    <mergeCell ref="A33:A45"/>
+    <mergeCell ref="A62:A72"/>
+    <mergeCell ref="A20:A31"/>
+    <mergeCell ref="A47:A59"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="M6:M26"/>
+    <mergeCell ref="N50:O50"/>
+    <mergeCell ref="M51:M63"/>
+    <mergeCell ref="N27:O27"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B1" location="Sheet1!B4" tooltip="Jump to TOP CEO EVENT" display="TOP CEO EVENT" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="G1" location="Sheet1!G4" tooltip="Jump to ULTIMATE CEO EVENT" display="ULTIMATE CEO EVENT" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="M1" location="Sheet1!M4" tooltip="Jump to WARM UP EVENT" display="WARM UP EVENT" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="S1" location="Sheet1!M4" tooltip="Jump to WARM UP EVENT" display="WARM UP EVENT" xr:uid="{77C0127A-5B0E-5946-A03F-81E7B22F1B74}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="W16" formula="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>